<commit_message>
removed second, empty sheet from xlsx file.
</commit_message>
<xml_diff>
--- a/pcb/Seed3-DevKit-Eurorack-Rev1/production/manual-files-for-JLCPCB/Seed3-DevKit-Eurorack-Rev1_bom.xlsx
+++ b/pcb/Seed3-DevKit-Eurorack-Rev1/production/manual-files-for-JLCPCB/Seed3-DevKit-Eurorack-Rev1_bom.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shensley\Documents\Github\ES-Seed3-DevKit-Eurorack\pcb\Seed3-DevKit-Eurorack-Rev1\production\manual-files-for-JLCPCB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA806A2C-E937-40C1-B2AC-CF1B77C5E2E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98966573-E6BF-4B74-AB11-8BD617EA2D63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-29040" yWindow="12315" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Seed3-DevKit-Eurorack-Rev1_bom" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seed3-DevKit-Eurorack-Rev1_bom'!$A$1:$C$42</definedName>
@@ -1663,13 +1662,4 @@
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>